<commit_message>
Fix completed application form formatting
</commit_message>
<xml_diff>
--- a/Prijavnica_ParKING.xlsx
+++ b/Prijavnica_ParKING.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List1" sheetId="1" r:id="R843490ffa6644fa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List1" sheetId="1" r:id="R59d29d0622b4439c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,6 +19,186 @@
     <x:t xml:space="preserve">Opće informacije o projektu</x:t>
   </x:si>
   <x:si>
+    <x:r>
+      <x:rPr>
+        <x:i/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">Kratki opis projekta </x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:b/>
+        <x:i/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">gdje je potrebno navesti</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:i/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">:</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">
+Ovaj projekt je namijenjen za …
+Aplikacija može biti korisna ili primijenjena za ..
+Zadatak ili problem koji se rješava je …
+</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:b/>
+        <x:i/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">Obavezno je navesti:</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">
+Aplikacija je pisana u</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:b/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve"> programskom jeziku (i razvojnom okruženju) </x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">…
+Aplikacija koristi bazu podataka … (</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:b/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">koju implementaciju: MS Access, MySQL, PostgreSQL, itd</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">)
+Ključne funkcionalnosti aplikacije </x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:b/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">po korisničkim ulogama odnosno vrstama korisnika</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve"> su</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:b/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">:</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">
+</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:b/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">- obični ili neregistrirani korisnik: ...
+- administrator: ...
+- registrirani korisnik: ...
+- korisnik s posebnim ovlastima: ...
+</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">
+</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:b/>
+        <x:sz val="11"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+        <x:scheme val="minor"/>
+      </x:rPr>
+      <x:t xml:space="preserve">Važno! Prijavnica se nastavniku šalje na pregled i odobrenje samo ukoliko suma bodova po odabranim funkcionalnostima iznosi minimalno 51 bod!</x:t>
+    </x:r>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">Funkcionalnosti aplikacije</x:t>
   </x:si>
   <x:si>
@@ -46,10 +226,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -57,7 +233,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -69,7 +245,7 @@
     <x:r>
       <x:rPr>
         <x:b/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -80,7 +256,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -94,10 +270,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -105,8 +277,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
+        <x:sz val="11"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -115,8 +286,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
+        <x:sz val="11"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -128,8 +298,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
+        <x:sz val="11"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -142,10 +311,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -153,8 +318,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
+        <x:sz val="11"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -163,8 +327,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
+        <x:sz val="11"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -176,8 +339,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
+        <x:sz val="11"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -186,8 +348,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
+        <x:sz val="11"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -201,10 +362,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Za svaki od pristupa (INI i/ili Windows registar) treba opisati:
 </x:t>
     </x:r>
@@ -212,7 +369,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -223,7 +380,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -238,10 +395,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Za svaki od pristupa (XML i/ili JSON) treba opisati:
 </x:t>
     </x:r>
@@ -249,7 +402,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -261,7 +414,7 @@
     <x:r>
       <x:rPr>
         <x:b/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -271,7 +424,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -287,10 +440,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -298,7 +447,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -311,7 +460,7 @@
     <x:r>
       <x:rPr>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -326,10 +475,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -337,7 +482,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -348,7 +493,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -361,7 +506,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -371,7 +516,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -386,10 +531,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -397,7 +538,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -414,10 +555,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -425,7 +562,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -439,10 +576,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -450,7 +583,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -466,10 +599,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -477,7 +606,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -487,7 +616,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -500,7 +629,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -511,7 +640,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -526,10 +655,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -537,7 +662,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -551,10 +676,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Za svaki korišteni mehanizam međusobnog zaključavanja treba opisati:
 </x:t>
     </x:r>
@@ -562,7 +683,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -576,10 +697,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -587,7 +704,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -597,7 +714,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -610,7 +727,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -624,10 +741,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -635,7 +748,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -653,10 +766,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -664,7 +773,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -679,10 +788,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -690,7 +795,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -704,10 +809,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -715,7 +816,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -730,10 +831,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -741,7 +838,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -755,10 +852,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -766,7 +859,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -782,10 +875,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -793,7 +882,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -807,10 +896,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -818,7 +903,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -829,7 +914,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -846,10 +931,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -857,7 +938,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -869,7 +950,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -882,7 +963,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -896,10 +977,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -907,7 +984,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -922,10 +999,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -933,7 +1006,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -948,10 +1021,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -959,7 +1028,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -974,10 +1043,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -985,7 +1050,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -999,10 +1064,6 @@
   </x:si>
   <x:si>
     <x:r>
-      <x:rPr>
-        <x:sz val="1100"/>
-        <x:color rgb="FF000000"/>
-      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -1010,7 +1071,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="1100"/>
+        <x:sz val="11"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -1030,7 +1091,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="13">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -1105,6 +1166,18 @@
       <x:sz val="11"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFF0000"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
   <x:fills count="4">
     <x:fill>
@@ -1353,7 +1426,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="106">
+  <x:cellXfs count="90">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -1552,8 +1625,14 @@
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -1561,108 +1640,56 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="3">
@@ -1870,7 +1897,7 @@
   <x:cols>
     <x:col min="1" max="1" width="6" customWidth="1"/>
     <x:col min="9" max="9" width="7.7109375" customWidth="1"/>
-    <x:col min="20" max="20" width="46" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="58" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" customHeight="1">
@@ -1988,164 +2015,157 @@
       <x:c r="S6" s="28"/>
     </x:row>
     <x:row r="7" ht="15" customHeight="1">
-      <x:c r="A7" s="68" t="str">
-        <x:v>ParKING je web aplikacija razvijena u Python Flask frameworku koja korisnicima omogućuje oglašavanje i rezervaciju privatnih parkirnih mjesta. Korisnici mogu registrirati račun, prijaviti se, objaviti vlastito parkirno mjesto, pregledavati i filtrirati dostupna mjesta te rezervirati tuđa parkirna mjesta. Administrator može upravljati korisnicima i rezervacijama te INI postavkama aplikacije. Aplikacija koristi SQLite bazu podataka, JSON datoteku za korisničke bilješke, hrvatsko/englesko sučelje, SQLAlchemy ORM i pokreće se u Docker containeru.</x:v>
-      </x:c>
-      <x:c r="B7" s="68"/>
-      <x:c r="C7" s="68"/>
-      <x:c r="D7" s="68"/>
-      <x:c r="E7" s="68"/>
-      <x:c r="F7" s="68"/>
-      <x:c r="G7" s="68"/>
-      <x:c r="H7" s="68"/>
-      <x:c r="I7" s="68"/>
-      <x:c r="J7" s="68"/>
-      <x:c r="K7" s="68"/>
-      <x:c r="L7" s="68"/>
-      <x:c r="M7" s="68"/>
-      <x:c r="N7" s="68"/>
-      <x:c r="O7" s="68"/>
-      <x:c r="P7" s="68"/>
-      <x:c r="Q7" s="68"/>
-      <x:c r="R7" s="68"/>
-      <x:c r="S7" s="68"/>
-      <x:c r="T7" s="71"/>
+      <x:c r="A7" s="29" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="29"/>
+      <x:c r="C7" s="29"/>
+      <x:c r="D7" s="29"/>
+      <x:c r="E7" s="29"/>
+      <x:c r="F7" s="29"/>
+      <x:c r="G7" s="29"/>
+      <x:c r="H7" s="29"/>
+      <x:c r="I7" s="29"/>
+      <x:c r="J7" s="29"/>
+      <x:c r="K7" s="29"/>
+      <x:c r="L7" s="29"/>
+      <x:c r="M7" s="29"/>
+      <x:c r="N7" s="29"/>
+      <x:c r="O7" s="29"/>
+      <x:c r="P7" s="29"/>
+      <x:c r="Q7" s="29"/>
+      <x:c r="R7" s="29"/>
+      <x:c r="S7" s="29"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="68"/>
-      <x:c r="B8" s="68"/>
-      <x:c r="C8" s="68"/>
-      <x:c r="D8" s="68"/>
-      <x:c r="E8" s="68"/>
-      <x:c r="F8" s="68"/>
-      <x:c r="G8" s="68"/>
-      <x:c r="H8" s="68"/>
-      <x:c r="I8" s="68"/>
-      <x:c r="J8" s="68"/>
-      <x:c r="K8" s="68"/>
-      <x:c r="L8" s="68"/>
-      <x:c r="M8" s="68"/>
-      <x:c r="N8" s="68"/>
-      <x:c r="O8" s="68"/>
-      <x:c r="P8" s="68"/>
-      <x:c r="Q8" s="68"/>
-      <x:c r="R8" s="68"/>
-      <x:c r="S8" s="68"/>
-      <x:c r="T8" s="71"/>
+      <x:c r="A8" s="29"/>
+      <x:c r="B8" s="29"/>
+      <x:c r="C8" s="29"/>
+      <x:c r="D8" s="29"/>
+      <x:c r="E8" s="29"/>
+      <x:c r="F8" s="29"/>
+      <x:c r="G8" s="29"/>
+      <x:c r="H8" s="29"/>
+      <x:c r="I8" s="29"/>
+      <x:c r="J8" s="29"/>
+      <x:c r="K8" s="29"/>
+      <x:c r="L8" s="29"/>
+      <x:c r="M8" s="29"/>
+      <x:c r="N8" s="29"/>
+      <x:c r="O8" s="29"/>
+      <x:c r="P8" s="29"/>
+      <x:c r="Q8" s="29"/>
+      <x:c r="R8" s="29"/>
+      <x:c r="S8" s="29"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="68"/>
-      <x:c r="B9" s="68"/>
-      <x:c r="C9" s="68"/>
-      <x:c r="D9" s="68"/>
-      <x:c r="E9" s="68"/>
-      <x:c r="F9" s="68"/>
-      <x:c r="G9" s="68"/>
-      <x:c r="H9" s="68"/>
-      <x:c r="I9" s="68"/>
-      <x:c r="J9" s="68"/>
-      <x:c r="K9" s="68"/>
-      <x:c r="L9" s="68"/>
-      <x:c r="M9" s="68"/>
-      <x:c r="N9" s="68"/>
-      <x:c r="O9" s="68"/>
-      <x:c r="P9" s="68"/>
-      <x:c r="Q9" s="68"/>
-      <x:c r="R9" s="68"/>
-      <x:c r="S9" s="68"/>
-      <x:c r="T9" s="71"/>
+      <x:c r="A9" s="29"/>
+      <x:c r="B9" s="29"/>
+      <x:c r="C9" s="29"/>
+      <x:c r="D9" s="29"/>
+      <x:c r="E9" s="29"/>
+      <x:c r="F9" s="29"/>
+      <x:c r="G9" s="29"/>
+      <x:c r="H9" s="29"/>
+      <x:c r="I9" s="29"/>
+      <x:c r="J9" s="29"/>
+      <x:c r="K9" s="29"/>
+      <x:c r="L9" s="29"/>
+      <x:c r="M9" s="29"/>
+      <x:c r="N9" s="29"/>
+      <x:c r="O9" s="29"/>
+      <x:c r="P9" s="29"/>
+      <x:c r="Q9" s="29"/>
+      <x:c r="R9" s="29"/>
+      <x:c r="S9" s="29"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="68"/>
-      <x:c r="B10" s="68"/>
-      <x:c r="C10" s="68"/>
-      <x:c r="D10" s="68"/>
-      <x:c r="E10" s="68"/>
-      <x:c r="F10" s="68"/>
-      <x:c r="G10" s="68"/>
-      <x:c r="H10" s="68"/>
-      <x:c r="I10" s="68"/>
-      <x:c r="J10" s="68"/>
-      <x:c r="K10" s="68"/>
-      <x:c r="L10" s="68"/>
-      <x:c r="M10" s="68"/>
-      <x:c r="N10" s="68"/>
-      <x:c r="O10" s="68"/>
-      <x:c r="P10" s="68"/>
-      <x:c r="Q10" s="68"/>
-      <x:c r="R10" s="68"/>
-      <x:c r="S10" s="68"/>
-      <x:c r="T10" s="71"/>
+      <x:c r="A10" s="29"/>
+      <x:c r="B10" s="29"/>
+      <x:c r="C10" s="29"/>
+      <x:c r="D10" s="29"/>
+      <x:c r="E10" s="29"/>
+      <x:c r="F10" s="29"/>
+      <x:c r="G10" s="29"/>
+      <x:c r="H10" s="29"/>
+      <x:c r="I10" s="29"/>
+      <x:c r="J10" s="29"/>
+      <x:c r="K10" s="29"/>
+      <x:c r="L10" s="29"/>
+      <x:c r="M10" s="29"/>
+      <x:c r="N10" s="29"/>
+      <x:c r="O10" s="29"/>
+      <x:c r="P10" s="29"/>
+      <x:c r="Q10" s="29"/>
+      <x:c r="R10" s="29"/>
+      <x:c r="S10" s="29"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="68"/>
-      <x:c r="B11" s="68"/>
-      <x:c r="C11" s="68"/>
-      <x:c r="D11" s="68"/>
-      <x:c r="E11" s="68"/>
-      <x:c r="F11" s="68"/>
-      <x:c r="G11" s="68"/>
-      <x:c r="H11" s="68"/>
-      <x:c r="I11" s="68"/>
-      <x:c r="J11" s="68"/>
-      <x:c r="K11" s="68"/>
-      <x:c r="L11" s="68"/>
-      <x:c r="M11" s="68"/>
-      <x:c r="N11" s="68"/>
-      <x:c r="O11" s="68"/>
-      <x:c r="P11" s="68"/>
-      <x:c r="Q11" s="68"/>
-      <x:c r="R11" s="68"/>
-      <x:c r="S11" s="68"/>
-      <x:c r="T11" s="71"/>
+      <x:c r="A11" s="29"/>
+      <x:c r="B11" s="29"/>
+      <x:c r="C11" s="29"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="29"/>
+      <x:c r="H11" s="29"/>
+      <x:c r="I11" s="29"/>
+      <x:c r="J11" s="29"/>
+      <x:c r="K11" s="29"/>
+      <x:c r="L11" s="29"/>
+      <x:c r="M11" s="29"/>
+      <x:c r="N11" s="29"/>
+      <x:c r="O11" s="29"/>
+      <x:c r="P11" s="29"/>
+      <x:c r="Q11" s="29"/>
+      <x:c r="R11" s="29"/>
+      <x:c r="S11" s="29"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="68"/>
-      <x:c r="B12" s="68"/>
-      <x:c r="C12" s="68"/>
-      <x:c r="D12" s="68"/>
-      <x:c r="E12" s="68"/>
-      <x:c r="F12" s="68"/>
-      <x:c r="G12" s="68"/>
-      <x:c r="H12" s="68"/>
-      <x:c r="I12" s="68"/>
-      <x:c r="J12" s="68"/>
-      <x:c r="K12" s="68"/>
-      <x:c r="L12" s="68"/>
-      <x:c r="M12" s="68"/>
-      <x:c r="N12" s="68"/>
-      <x:c r="O12" s="68"/>
-      <x:c r="P12" s="68"/>
-      <x:c r="Q12" s="68"/>
-      <x:c r="R12" s="68"/>
-      <x:c r="S12" s="68"/>
-      <x:c r="T12" s="71"/>
+      <x:c r="A12" s="29"/>
+      <x:c r="B12" s="29"/>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="29"/>
+      <x:c r="G12" s="29"/>
+      <x:c r="H12" s="29"/>
+      <x:c r="I12" s="29"/>
+      <x:c r="J12" s="29"/>
+      <x:c r="K12" s="29"/>
+      <x:c r="L12" s="29"/>
+      <x:c r="M12" s="29"/>
+      <x:c r="N12" s="29"/>
+      <x:c r="O12" s="29"/>
+      <x:c r="P12" s="29"/>
+      <x:c r="Q12" s="29"/>
+      <x:c r="R12" s="29"/>
+      <x:c r="S12" s="29"/>
     </x:row>
     <x:row r="13" ht="122.25" customHeight="1">
-      <x:c r="A13" s="68"/>
-      <x:c r="B13" s="68"/>
-      <x:c r="C13" s="68"/>
-      <x:c r="D13" s="68"/>
-      <x:c r="E13" s="68"/>
-      <x:c r="F13" s="68"/>
-      <x:c r="G13" s="68"/>
-      <x:c r="H13" s="68"/>
-      <x:c r="I13" s="68"/>
-      <x:c r="J13" s="68"/>
-      <x:c r="K13" s="68"/>
-      <x:c r="L13" s="68"/>
-      <x:c r="M13" s="68"/>
-      <x:c r="N13" s="68"/>
-      <x:c r="O13" s="68"/>
-      <x:c r="P13" s="68"/>
-      <x:c r="Q13" s="68"/>
-      <x:c r="R13" s="68"/>
-      <x:c r="S13" s="68"/>
-      <x:c r="T13" s="71"/>
+      <x:c r="A13" s="29"/>
+      <x:c r="B13" s="29"/>
+      <x:c r="C13" s="29"/>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="29"/>
+      <x:c r="H13" s="29"/>
+      <x:c r="I13" s="29"/>
+      <x:c r="J13" s="29"/>
+      <x:c r="K13" s="29"/>
+      <x:c r="L13" s="29"/>
+      <x:c r="M13" s="29"/>
+      <x:c r="N13" s="29"/>
+      <x:c r="O13" s="29"/>
+      <x:c r="P13" s="29"/>
+      <x:c r="Q13" s="29"/>
+      <x:c r="R13" s="29"/>
+      <x:c r="S13" s="29"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="28" t="s">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B15" s="28"/>
       <x:c r="C15" s="28"/>
@@ -2168,7 +2188,7 @@
     </x:row>
     <x:row r="16" ht="15" customHeight="1">
       <x:c r="A16" s="30" t="s">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B16" s="30"/>
       <x:c r="C16" s="30"/>
@@ -2212,10 +2232,10 @@
     </x:row>
     <x:row r="18" ht="43.150001525878906" customHeight="1">
       <x:c r="A18" s="5" t="s">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B18" s="31" t="s">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C18" s="31"/>
       <x:c r="D18" s="31"/>
@@ -2224,10 +2244,10 @@
       <x:c r="G18" s="31"/>
       <x:c r="H18" s="31"/>
       <x:c r="I18" s="6" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J18" s="32" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="K18" s="32"/>
       <x:c r="L18" s="32"/>
@@ -2238,8 +2258,8 @@
       <x:c r="Q18" s="32"/>
       <x:c r="R18" s="32"/>
       <x:c r="S18" s="32"/>
-      <x:c r="T18" s="15" t="s">
-        <x:v>9</x:v>
+      <x:c r="T18" s="89" t="s">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="U18" s="15"/>
       <x:c r="V18" s="15"/>
@@ -2251,12 +2271,12 @@
       <x:c r="AB18" s="15"/>
       <x:c r="AC18" s="15"/>
     </x:row>
-    <x:row r="19" ht="100" customHeight="1">
+    <x:row r="19" ht="88" customHeight="1">
       <x:c r="A19" s="3">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B19" s="12" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C19" s="13"/>
       <x:c r="D19" s="13"/>
@@ -2268,7 +2288,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J19" s="12" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="K19" s="13"/>
       <x:c r="L19" s="13"/>
@@ -2279,7 +2299,7 @@
       <x:c r="Q19" s="13"/>
       <x:c r="R19" s="13"/>
       <x:c r="S19" s="14"/>
-      <x:c r="T19" s="74" t="str">
+      <x:c r="T19" s="82" t="str">
         <x:v>Implementirane su tri korisničke klase: User, ParkingSpot i Reservation.
 User: atributi id, username, password_hash, role; metode set_password(), check_password(), is_admin().
 ParkingSpot: atributi id, owner_id, name, location, price_per_hour, description; metode display_price(), is_owned_by().
@@ -2296,12 +2316,12 @@
       <x:c r="AB19" s="13"/>
       <x:c r="AC19" s="14"/>
     </x:row>
-    <x:row r="20" ht="100" customHeight="1">
+    <x:row r="20" ht="82" customHeight="1">
       <x:c r="A20" s="3">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="24" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C20" s="25"/>
       <x:c r="D20" s="25"/>
@@ -2313,7 +2333,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J20" s="33" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="K20" s="34"/>
       <x:c r="L20" s="34"/>
@@ -2324,7 +2344,7 @@
       <x:c r="Q20" s="34"/>
       <x:c r="R20" s="34"/>
       <x:c r="S20" s="35"/>
-      <x:c r="T20" s="74" t="str">
+      <x:c r="T20" s="82" t="str">
         <x:v>Aplikacija sadrži više od tri web forme/dijaloga: prijava, registracija, popis parkinga, dodavanje/uređivanje parkinga, detalji parkinga, rezervacija, moje rezervacije te administratorske forme za korisnike i rezervacije.
 Komunikacija među formama demonstrira se npr. odabirom parkinga na popisu ili detaljima, čime se njegov parking_id prenosi na formu za rezervaciju; nakon spremanja korisnik se preusmjerava na pregled svojih rezervacija.</x:v>
       </x:c>
@@ -2338,12 +2358,12 @@
       <x:c r="AB20" s="13"/>
       <x:c r="AC20" s="14"/>
     </x:row>
-    <x:row r="21" ht="80.25" customHeight="1">
+    <x:row r="21" ht="80" customHeight="1">
       <x:c r="A21" s="3">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B21" s="12" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C21" s="13"/>
       <x:c r="D21" s="13"/>
@@ -2355,7 +2375,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J21" s="33" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="K21" s="34"/>
       <x:c r="L21" s="34"/>
@@ -2366,7 +2386,7 @@
       <x:c r="Q21" s="34"/>
       <x:c r="R21" s="34"/>
       <x:c r="S21" s="35"/>
-      <x:c r="T21" s="12" t="str">
+      <x:c r="T21" s="82" t="str">
         <x:v>Aplikacija podržava hrvatsko i englesko korisničko sučelje. Jezik se može promijeniti tijekom rada aplikacije pomoću HR/EN poveznica u navigaciji bez izlaska iz aplikacije.
 Prevedeno je više od 5 dijaloga/stranica: prijava, registracija, popis parkinga, moji parkinzi, forma za dodavanje/uređivanje parkinga, detalji parkinga, forma rezervacije, moje rezervacije, JSON bilješke i INI postavke.</x:v>
       </x:c>
@@ -2380,12 +2400,12 @@
       <x:c r="AB21" s="13"/>
       <x:c r="AC21" s="14"/>
     </x:row>
-    <x:row r="22" ht="82.9000015258789" customHeight="1">
+    <x:row r="22" ht="74" customHeight="1">
       <x:c r="A22" s="3">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B22" s="24" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C22" s="25"/>
       <x:c r="D22" s="25"/>
@@ -2397,7 +2417,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J22" s="12" t="s">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="K22" s="13"/>
       <x:c r="L22" s="13"/>
@@ -2408,7 +2428,7 @@
       <x:c r="Q22" s="13"/>
       <x:c r="R22" s="13"/>
       <x:c r="S22" s="14"/>
-      <x:c r="T22" s="12" t="str">
+      <x:c r="T22" s="82" t="str">
         <x:v>Postavke aplikacije spremaju se i učitavaju iz INI datoteke config.ini pomoću Python modula configparser.
 Spremaju se najmanje dvije postavke: default_language (zadani jezik HR/EN) i items_per_page (broj parkinga prikazanih po stranici). Administrator ih može mijenjati kroz stranicu Postavke, a promjene se zapisuju natrag u config.ini.</x:v>
       </x:c>
@@ -2422,12 +2442,12 @@
       <x:c r="AB22" s="13"/>
       <x:c r="AC22" s="14"/>
     </x:row>
-    <x:row r="23" ht="122.44999694824219" customHeight="1">
+    <x:row r="23" ht="82" customHeight="1">
       <x:c r="A23" s="3">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B23" s="24" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C23" s="25"/>
       <x:c r="D23" s="25"/>
@@ -2439,7 +2459,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="J23" s="12" t="s">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="K23" s="13"/>
       <x:c r="L23" s="13"/>
@@ -2450,7 +2470,7 @@
       <x:c r="Q23" s="13"/>
       <x:c r="R23" s="13"/>
       <x:c r="S23" s="14"/>
-      <x:c r="T23" s="12" t="str">
+      <x:c r="T23" s="82" t="str">
         <x:v>Aplikacija koristi JSON datoteku data/parking_notes.json za niz korisničkih bilješki. Svaki zapis sadrži id, user_id, title i text.
 Podržane su sve CRUD operacije: čitanje popisa i pojedine bilješke, dodavanje nove bilješke, uređivanje naslova/teksta te brisanje bilješke. Operacije su implementirane u modulu json_store.py i dostupne kroz web sučelje Bilješke.</x:v>
       </x:c>
@@ -2464,12 +2484,12 @@
       <x:c r="AB23" s="13"/>
       <x:c r="AC23" s="14"/>
     </x:row>
-    <x:row r="24" ht="82" customHeight="1">
+    <x:row r="24" ht="80" customHeight="1">
       <x:c r="A24" s="3">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B24" s="24" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C24" s="25"/>
       <x:c r="D24" s="25"/>
@@ -2481,7 +2501,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J24" s="12" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="K24" s="13"/>
       <x:c r="L24" s="13"/>
@@ -2492,7 +2512,7 @@
       <x:c r="Q24" s="13"/>
       <x:c r="R24" s="13"/>
       <x:c r="S24" s="14"/>
-      <x:c r="T24" s="73" t="str">
+      <x:c r="T24" s="82" t="str">
         <x:v>Aplikacija koristi vlastiti binarni format datoteke data/search_history.bin za pohranu niza zapisa povijesti pretraga. Datoteka ima vlastito zaglavlje PKSR, verziju formata i broj zapisa. Svaki binarni zapis sadrži user_id, vrijeme zapisa, maksimalnu cijenu i lokaciju promjenjive duljine. Implementirane su funkcije za zapis cijelog niza u binarnu datoteku i ponovno čitanje zapisa iz tog formata. Binarni sadržaj demonstriran je alatom xxd, pri čemu se vidi zaglavlje PKSR i strukturirani binarni podaci, a ne tekstualni zapis.</x:v>
       </x:c>
       <x:c r="U24" s="13"/>
@@ -2505,12 +2525,12 @@
       <x:c r="AB24" s="13"/>
       <x:c r="AC24" s="14"/>
     </x:row>
-    <x:row r="25" ht="100" customHeight="1">
+    <x:row r="25" ht="82" customHeight="1">
       <x:c r="A25" s="3">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B25" s="24" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C25" s="25"/>
       <x:c r="D25" s="25"/>
@@ -2522,7 +2542,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="J25" s="12" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="K25" s="13"/>
       <x:c r="L25" s="13"/>
@@ -2533,7 +2553,7 @@
       <x:c r="Q25" s="13"/>
       <x:c r="R25" s="13"/>
       <x:c r="S25" s="14"/>
-      <x:c r="T25" s="74" t="str">
+      <x:c r="T25" s="82" t="str">
         <x:v>Aplikacija koristi SQLite bazu podataka preko SQLAlchemy ORM-a. Baza služi za trajnu pohranu korisnika, parkirnih mjesta i rezervacija.
 Tablice: users, parking_spots i reservations. Nad sve tri tablice demonstriraju se operacije čitanja, dodavanja, uređivanja i brisanja. Korisnik upravlja vlastitim parkirnim mjestima i rezervacijama, a administrator kroz administratorsko sučelje upravlja korisnicima i rezervacijama.</x:v>
       </x:c>
@@ -2547,12 +2567,12 @@
       <x:c r="AB25" s="13"/>
       <x:c r="AC25" s="14"/>
     </x:row>
-    <x:row r="26" ht="100" customHeight="1">
+    <x:row r="26" ht="80" customHeight="1">
       <x:c r="A26" s="3">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B26" s="24" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C26" s="25"/>
       <x:c r="D26" s="25"/>
@@ -2564,7 +2584,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J26" s="12" t="s">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="K26" s="13"/>
       <x:c r="L26" s="13"/>
@@ -2575,7 +2595,7 @@
       <x:c r="Q26" s="13"/>
       <x:c r="R26" s="13"/>
       <x:c r="S26" s="14"/>
-      <x:c r="T26" s="74" t="str">
+      <x:c r="T26" s="82" t="str">
         <x:v>Sortiranje i filtriranje provodi se nad zapisima tablice parking_spots. Parkirna mjesta mogu se filtrirati po lokaciji te sortirati po cijeni uzlazno/silazno i po nazivu.
 Izračunato polje: ukupna cijena rezervacije računa se metodom Reservation.total_price() iz trajanja rezervacije i cijene parkinga po satu.
 Lookup/povezana polja ostvarena su SQLAlchemy relacijama, npr. Reservation.parking za dohvat naziva i lokacije parkinga te ParkingSpot.owner za dohvat vlasnika.</x:v>
@@ -2590,12 +2610,12 @@
       <x:c r="AB26" s="13"/>
       <x:c r="AC26" s="14"/>
     </x:row>
-    <x:row r="27" ht="70" customHeight="1">
+    <x:row r="27" ht="78" customHeight="1">
       <x:c r="A27" s="3">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B27" s="12" t="s">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C27" s="13"/>
       <x:c r="D27" s="13"/>
@@ -2607,7 +2627,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J27" s="10" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="K27" s="10"/>
       <x:c r="L27" s="10"/>
@@ -2618,7 +2638,7 @@
       <x:c r="Q27" s="10"/>
       <x:c r="R27" s="10"/>
       <x:c r="S27" s="10"/>
-      <x:c r="T27" s="85" t="str">
+      <x:c r="T27" s="83" t="str">
         <x:v>Tablica parking_spots sadrži BLOB polje photo u koje se sprema fotografija parkirnog mjesta kao binarni sadržaj. Uz njega se sprema i MIME tip slike (photo_mime). Fotografija se učitava kroz obrazac za dodavanje/uređivanje parkinga, sprema izravno u SQLite bazu, može se zamijeniti ili ukloniti te se čita iz baze i prikazuje na stranici detalja parkinga. Podržani su JPEG, PNG i WebP formati uz ograničenje veličine datoteke.</x:v>
       </x:c>
       <x:c r="U27" s="10"/>
@@ -2631,12 +2651,12 @@
       <x:c r="AB27" s="10"/>
       <x:c r="AC27" s="10"/>
     </x:row>
-    <x:row r="28" ht="70" customHeight="1">
+    <x:row r="28" ht="86" customHeight="1">
       <x:c r="A28" s="3">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B28" s="24" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C28" s="25"/>
       <x:c r="D28" s="25"/>
@@ -2648,7 +2668,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J28" s="10" t="s">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K28" s="10"/>
       <x:c r="L28" s="10"/>
@@ -2659,7 +2679,7 @@
       <x:c r="Q28" s="10"/>
       <x:c r="R28" s="10"/>
       <x:c r="S28" s="10"/>
-      <x:c r="T28" s="85" t="str">
+      <x:c r="T28" s="83" t="str">
         <x:v>Aplikacija automatski generira PDF potvrdu rezervacije. Izvještaj sadrži podatke o rezervaciji: identifikator, početak i završetak, trajanje, status i izračunatu ukupnu cijenu. U PDF se uključuju i povezani podaci iz tablice users (korisničko ime korisnika) te iz tablice parking_spots (naziv parkinga, lokacija, vlasnik i cijena po satu), čime se demonstrira master-detail izvještaj nad više tablica. PDF se generira pomoću biblioteke ReportLab i korisnik ga može preuzeti iz popisa svojih rezervacija.</x:v>
       </x:c>
       <x:c r="U28" s="10"/>
@@ -2672,12 +2692,12 @@
       <x:c r="AB28" s="10"/>
       <x:c r="AC28" s="10"/>
     </x:row>
-    <x:row r="29" ht="78" customHeight="1">
+    <x:row r="29" ht="90" customHeight="1">
       <x:c r="A29" s="3">
         <x:v>11</x:v>
       </x:c>
       <x:c r="B29" s="24" t="s">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C29" s="25"/>
       <x:c r="D29" s="25"/>
@@ -2689,7 +2709,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J29" s="10" t="s">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="K29" s="11"/>
       <x:c r="L29" s="11"/>
@@ -2700,7 +2720,7 @@
       <x:c r="Q29" s="11"/>
       <x:c r="R29" s="11"/>
       <x:c r="S29" s="11"/>
-      <x:c r="T29" s="85" t="str">
+      <x:c r="T29" s="83" t="str">
         <x:v>Aplikacija demonstrira paralelno izvršavanje tri neovisna mrežna zadatka pomoću bazena dretvi (concurrent.futures.ThreadPoolExecutor). Paralelno se dohvaćaju vremenski podaci za Zagreb, Samobor i Veliku Goricu s udaljenog REST servisa Open-Meteo. Administratorska stranica Dretve prikazuje naziv dretve koja je izvršila svaki zadatak te uspoređuje ukupno vrijeme sekvencijalnog i paralelnog izvršavanja i izračunava faktor ubrzanja. Korištenje više dretvi smanjuje ukupno čekanje jer se mrežni I/O zahtjevi izvršavaju istodobno.</x:v>
       </x:c>
       <x:c r="U29" s="11"/>
@@ -2718,7 +2738,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B30" s="24" t="s">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C30" s="25"/>
       <x:c r="D30" s="25"/>
@@ -2730,7 +2750,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J30" s="10" t="s">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="K30" s="10"/>
       <x:c r="L30" s="10"/>
@@ -2741,7 +2761,7 @@
       <x:c r="Q30" s="10"/>
       <x:c r="R30" s="10"/>
       <x:c r="S30" s="10"/>
-      <x:c r="T30" s="85"/>
+      <x:c r="T30" s="83"/>
       <x:c r="U30" s="10"/>
       <x:c r="V30" s="10"/>
       <x:c r="W30" s="10"/>
@@ -2752,12 +2772,12 @@
       <x:c r="AB30" s="10"/>
       <x:c r="AC30" s="10"/>
     </x:row>
-    <x:row r="31" ht="62" customHeight="1">
+    <x:row r="31" ht="68" customHeight="1">
       <x:c r="A31" s="3">
         <x:v>13</x:v>
       </x:c>
       <x:c r="B31" s="24" t="s">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C31" s="25"/>
       <x:c r="D31" s="25"/>
@@ -2769,7 +2789,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J31" s="10" t="s">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="K31" s="10"/>
       <x:c r="L31" s="10"/>
@@ -2780,7 +2800,7 @@
       <x:c r="Q31" s="10"/>
       <x:c r="R31" s="10"/>
       <x:c r="S31" s="10"/>
-      <x:c r="T31" s="85" t="str">
+      <x:c r="T31" s="83" t="str">
         <x:v>Za zaštitu zajedničkog zapisnika zahtjeva koji istodobno koriste radne dretve koristi se threading.Lock. Svaka dretva prije upisa rezultata u zajedničku strukturu ulazi u kritični odsječak zaštićen Lock objektom, čime se sprječava istodobno nekontrolirano mijenjanje zajedničkih podataka.</x:v>
       </x:c>
       <x:c r="U31" s="10"/>
@@ -2793,12 +2813,12 @@
       <x:c r="AB31" s="10"/>
       <x:c r="AC31" s="10"/>
     </x:row>
-    <x:row r="32" ht="88" customHeight="1">
+    <x:row r="32" ht="94" customHeight="1">
       <x:c r="A32" s="3">
         <x:v>14</x:v>
       </x:c>
       <x:c r="B32" s="12" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C32" s="13"/>
       <x:c r="D32" s="13"/>
@@ -2810,7 +2830,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J32" s="10" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="K32" s="10"/>
       <x:c r="L32" s="10"/>
@@ -2821,7 +2841,7 @@
       <x:c r="Q32" s="10"/>
       <x:c r="R32" s="10"/>
       <x:c r="S32" s="10"/>
-      <x:c r="T32" s="85" t="str">
+      <x:c r="T32" s="83" t="str">
         <x:v>Aplikacija demonstrira komunikaciju između dva zasebna procesa. Proces A je Flask aplikacija (run.py) koja pomoću subprocess.run pokreće proces B, zasebnu Python skriptu reservation_worker.py. Proces B čita SQLite bazu i provjerava konzistentnost rezervacija, uključujući neispravne vremenske intervale i preklapanja aktivnih rezervacija. Proces B vraća cjelobrojni izlazni kod: 0 kada je provjera uspješna, 1 kada su pronađeni problemi u podacima, a 2 kod tehničke greške. Proces A čita returncode, stdout i stderr te korisniku prikazuje odgovarajuću poruku. Administratorska stranica Procesi omogućuje i kontroliranu simulaciju greške radi demonstracije nenultog izlaznog koda.</x:v>
       </x:c>
       <x:c r="U32" s="10"/>
@@ -2839,7 +2859,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B33" s="24" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C33" s="25"/>
       <x:c r="D33" s="25"/>
@@ -2851,7 +2871,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="J33" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K33" s="10"/>
       <x:c r="L33" s="10"/>
@@ -2862,7 +2882,7 @@
       <x:c r="Q33" s="10"/>
       <x:c r="R33" s="10"/>
       <x:c r="S33" s="10"/>
-      <x:c r="T33" s="85"/>
+      <x:c r="T33" s="83"/>
       <x:c r="U33" s="10"/>
       <x:c r="V33" s="10"/>
       <x:c r="W33" s="10"/>
@@ -2878,7 +2898,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B34" s="24" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C34" s="25"/>
       <x:c r="D34" s="25"/>
@@ -2890,7 +2910,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="J34" s="10" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K34" s="10"/>
       <x:c r="L34" s="10"/>
@@ -2901,7 +2921,7 @@
       <x:c r="Q34" s="10"/>
       <x:c r="R34" s="10"/>
       <x:c r="S34" s="10"/>
-      <x:c r="T34" s="85"/>
+      <x:c r="T34" s="83"/>
       <x:c r="U34" s="10"/>
       <x:c r="V34" s="10"/>
       <x:c r="W34" s="10"/>
@@ -2917,7 +2937,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B35" s="24" t="s">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C35" s="25"/>
       <x:c r="D35" s="25"/>
@@ -2929,7 +2949,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J35" s="10" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="K35" s="10"/>
       <x:c r="L35" s="10"/>
@@ -2940,7 +2960,7 @@
       <x:c r="Q35" s="10"/>
       <x:c r="R35" s="10"/>
       <x:c r="S35" s="10"/>
-      <x:c r="T35" s="85"/>
+      <x:c r="T35" s="83"/>
       <x:c r="U35" s="10"/>
       <x:c r="V35" s="10"/>
       <x:c r="W35" s="10"/>
@@ -2956,7 +2976,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B36" s="24" t="s">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C36" s="25"/>
       <x:c r="D36" s="25"/>
@@ -2968,7 +2988,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J36" s="10" t="s">
-        <x:v>44</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="K36" s="10"/>
       <x:c r="L36" s="10"/>
@@ -2979,7 +2999,7 @@
       <x:c r="Q36" s="10"/>
       <x:c r="R36" s="10"/>
       <x:c r="S36" s="10"/>
-      <x:c r="T36" s="85"/>
+      <x:c r="T36" s="83"/>
       <x:c r="U36" s="10"/>
       <x:c r="V36" s="10"/>
       <x:c r="W36" s="10"/>
@@ -2995,7 +3015,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B37" s="24" t="s">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C37" s="25"/>
       <x:c r="D37" s="25"/>
@@ -3007,7 +3027,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="J37" s="10" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="K37" s="10"/>
       <x:c r="L37" s="10"/>
@@ -3018,7 +3038,7 @@
       <x:c r="Q37" s="10"/>
       <x:c r="R37" s="10"/>
       <x:c r="S37" s="10"/>
-      <x:c r="T37" s="85"/>
+      <x:c r="T37" s="83"/>
       <x:c r="U37" s="10"/>
       <x:c r="V37" s="10"/>
       <x:c r="W37" s="10"/>
@@ -3029,12 +3049,12 @@
       <x:c r="AB37" s="10"/>
       <x:c r="AC37" s="10"/>
     </x:row>
-    <x:row r="38" ht="70" customHeight="1">
+    <x:row r="38" ht="76" customHeight="1">
       <x:c r="A38" s="3">
         <x:v>20</x:v>
       </x:c>
       <x:c r="B38" s="24" t="s">
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C38" s="25"/>
       <x:c r="D38" s="25"/>
@@ -3046,7 +3066,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J38" s="10" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="K38" s="10"/>
       <x:c r="L38" s="10"/>
@@ -3057,7 +3077,7 @@
       <x:c r="Q38" s="10"/>
       <x:c r="R38" s="10"/>
       <x:c r="S38" s="10"/>
-      <x:c r="T38" s="85" t="str">
+      <x:c r="T38" s="83" t="str">
         <x:v>Aplikacija se spaja na udaljeni REST web servis Open-Meteo (https://open-meteo.com/). HTTP zahtjevima dohvaća aktualne vremenske podatke za tri lokacije: Zagreb, Samobor i Veliku Goricu. Podaci se koriste na administratorskoj demonstracijskoj stranici Dretve kako bi se prikazali rezultati udaljenog servisa i usporedile performanse sekvencijalnih i paralelnih mrežnih poziva.</x:v>
       </x:c>
       <x:c r="U38" s="10"/>
@@ -3070,12 +3090,12 @@
       <x:c r="AB38" s="10"/>
       <x:c r="AC38" s="10"/>
     </x:row>
-    <x:row r="39" ht="105" customHeight="1">
+    <x:row r="39" ht="110" customHeight="1">
       <x:c r="A39" s="3">
         <x:v>21</x:v>
       </x:c>
       <x:c r="B39" s="24" t="s">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C39" s="25"/>
       <x:c r="D39" s="25"/>
@@ -3087,7 +3107,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="J39" s="10" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="K39" s="10"/>
       <x:c r="L39" s="10"/>
@@ -3098,7 +3118,7 @@
       <x:c r="Q39" s="10"/>
       <x:c r="R39" s="10"/>
       <x:c r="S39" s="10"/>
-      <x:c r="T39" s="85" t="str">
+      <x:c r="T39" s="83" t="str">
         <x:v>Aplikacija sadrži REST klijent komponentu u glavnoj Flask aplikaciji (run.py, port 5000) koja se preko HTTP-a spaja na vlastiti ParKING REST servis implementiran kao zasebna Flask aplikacija (api_app.py, port 5001) i zaseban proces. Obje aplikacije rade u istom Docker containeru, ali imaju odvojene Flask instance i procese. Servis izlaže resurse /api/parkings i /api/reservations. Za parkings podržani su GET/POST te GET/PUT/DELETE nad pojedinim parkingom; za reservations GET/POST te GET/DELETE nad pojedinom rezervacijom. REST klijent demonstrira HTTP GET za oba resursa. Odvojenost se može dokazati tako da /api/parkings na portu 5001 vraća 401 bez Bearer tokena, dok ista ruta na portu 5000 vraća 404.</x:v>
       </x:c>
       <x:c r="U39" s="10"/>
@@ -3111,12 +3131,12 @@
       <x:c r="AB39" s="10"/>
       <x:c r="AC39" s="10"/>
     </x:row>
-    <x:row r="40" ht="105" customHeight="1">
+    <x:row r="40" ht="108" customHeight="1">
       <x:c r="A40" s="3">
         <x:v>22</x:v>
       </x:c>
       <x:c r="B40" s="12" t="s">
-        <x:v>51</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C40" s="13"/>
       <x:c r="D40" s="13"/>
@@ -3128,7 +3148,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J40" s="10" t="s">
-        <x:v>52</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="K40" s="10"/>
       <x:c r="L40" s="10"/>
@@ -3139,7 +3159,7 @@
       <x:c r="Q40" s="10"/>
       <x:c r="R40" s="10"/>
       <x:c r="S40" s="10"/>
-      <x:c r="T40" s="85" t="str">
+      <x:c r="T40" s="83" t="str">
         <x:v>Vlastiti REST servis koristi Bearer API token u HTTP zaglavlju Authorization. Zahtjev bez tokena ili s neispravnim tokenom vraća HTTP 401. Autorizacija se provodi po korisniku i ulozi. Na resursu /api/parkings obični korisnik može čitati parkinge, ali PUT/DELETE nad tuđim parkingom vraća HTTP 403; vlasnik parkinga i administrator imaju pravo izmjene. Na resursu /api/reservations obični korisnik vidi i dohvaća samo vlastite rezervacije, dok pokušaj pristupa tuđoj rezervaciji vraća HTTP 403; administrator ima pristup svim rezervacijama. Time se mogu demonstrirati dva korisnika (npr. gost i vlasnik/admin) i dva resursa (parkings i reservations) s različitim ovlastima.</x:v>
       </x:c>
       <x:c r="U40" s="10"/>
@@ -3157,7 +3177,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B41" s="24" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C41" s="25"/>
       <x:c r="D41" s="25"/>
@@ -3169,7 +3189,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J41" s="10" t="s">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="K41" s="10"/>
       <x:c r="L41" s="10"/>
@@ -3180,7 +3200,7 @@
       <x:c r="Q41" s="10"/>
       <x:c r="R41" s="10"/>
       <x:c r="S41" s="10"/>
-      <x:c r="T41" s="85" t="str">
+      <x:c r="T41" s="83" t="str">
         <x:v>Aplikacija demonstrira simetrično šifriranje i dešifriranje korisničkih bilješki pomoću algoritma AES-GCM. Za korisnika se generira šifrirana datoteka u direktoriju exports, s vlastitim zaglavljem PKAE i slučajnim nonceom. Šifrirani sadržaj nije čitljiv kao tekst, a aplikacija ga može dešifrirati i ponovno prikazati izvorne bilješke. Lozinke korisnika ne pohranjuju se reverzibilno šifrirane.</x:v>
       </x:c>
       <x:c r="U41" s="10"/>
@@ -3198,7 +3218,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B42" s="24" t="s">
-        <x:v>55</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C42" s="25"/>
       <x:c r="D42" s="25"/>
@@ -3210,7 +3230,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J42" s="10" t="s">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="K42" s="10"/>
       <x:c r="L42" s="10"/>
@@ -3221,7 +3241,7 @@
       <x:c r="Q42" s="10"/>
       <x:c r="R42" s="10"/>
       <x:c r="S42" s="10"/>
-      <x:c r="T42" s="10"/>
+      <x:c r="T42" s="83"/>
       <x:c r="U42" s="10"/>
       <x:c r="V42" s="10"/>
       <x:c r="W42" s="10"/>
@@ -3232,12 +3252,12 @@
       <x:c r="AB42" s="10"/>
       <x:c r="AC42" s="10"/>
     </x:row>
-    <x:row r="43" ht="88" customHeight="1">
+    <x:row r="43" ht="92" customHeight="1">
       <x:c r="A43" s="3">
         <x:v>25</x:v>
       </x:c>
       <x:c r="B43" s="24" t="s">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C43" s="25"/>
       <x:c r="D43" s="25"/>
@@ -3249,7 +3269,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="J43" s="10" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="K43" s="10"/>
       <x:c r="L43" s="10"/>
@@ -3260,7 +3280,7 @@
       <x:c r="Q43" s="10"/>
       <x:c r="R43" s="10"/>
       <x:c r="S43" s="10"/>
-      <x:c r="T43" s="85" t="str">
+      <x:c r="T43" s="83" t="str">
         <x:v>Aplikacija demonstrira SHA-256 funkciju sažimanja nad proizvoljnim tekstom. Koristi se promjenjiva sol koja se ne sprema u bazu ni datoteku, nego se deterministički izvodi po pravilu SHA256('ParKING-SHA256-salt:&lt;user_id&gt;:&lt;username&gt;')[0:16], pa različiti korisnici dobivaju različitu sol. Uz sol se koristi i papar iz raspona 0-255. Provjera ispravnosti papra demonstrira se prolaskom kroz cijeli raspon svih 256 mogućih vrijednosti; za testni sažetak pronađena je vrijednost papra 137 i potvrđena ispravnost sažetka.</x:v>
       </x:c>
       <x:c r="U43" s="10"/>
@@ -3278,7 +3298,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B44" s="24" t="s">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C44" s="25"/>
       <x:c r="D44" s="25"/>
@@ -3290,7 +3310,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J44" s="10" t="s">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="K44" s="10"/>
       <x:c r="L44" s="10"/>
@@ -3301,7 +3321,7 @@
       <x:c r="Q44" s="10"/>
       <x:c r="R44" s="10"/>
       <x:c r="S44" s="10"/>
-      <x:c r="T44" s="10"/>
+      <x:c r="T44" s="83"/>
       <x:c r="U44" s="10"/>
       <x:c r="V44" s="10"/>
       <x:c r="W44" s="10"/>
@@ -3317,7 +3337,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B45" s="24" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C45" s="25"/>
       <x:c r="D45" s="25"/>
@@ -3329,7 +3349,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J45" s="10" t="s">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="K45" s="10"/>
       <x:c r="L45" s="10"/>
@@ -3340,7 +3360,7 @@
       <x:c r="Q45" s="10"/>
       <x:c r="R45" s="10"/>
       <x:c r="S45" s="10"/>
-      <x:c r="T45" s="10"/>
+      <x:c r="T45" s="83"/>
       <x:c r="U45" s="10"/>
       <x:c r="V45" s="10"/>
       <x:c r="W45" s="10"/>
@@ -3356,7 +3376,7 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B46" s="24" t="s">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C46" s="25"/>
       <x:c r="D46" s="25"/>
@@ -3368,7 +3388,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J46" s="10" t="s">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="K46" s="10"/>
       <x:c r="L46" s="10"/>
@@ -3379,7 +3399,7 @@
       <x:c r="Q46" s="10"/>
       <x:c r="R46" s="10"/>
       <x:c r="S46" s="10"/>
-      <x:c r="T46" s="10"/>
+      <x:c r="T46" s="83"/>
       <x:c r="U46" s="10"/>
       <x:c r="V46" s="10"/>
       <x:c r="W46" s="10"/>
@@ -3395,7 +3415,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B47" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C47" s="13"/>
       <x:c r="D47" s="13"/>
@@ -3407,7 +3427,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J47" s="10" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="K47" s="10"/>
       <x:c r="L47" s="10"/>
@@ -3418,7 +3438,7 @@
       <x:c r="Q47" s="10"/>
       <x:c r="R47" s="10"/>
       <x:c r="S47" s="10"/>
-      <x:c r="T47" s="10"/>
+      <x:c r="T47" s="83"/>
       <x:c r="U47" s="10"/>
       <x:c r="V47" s="10"/>
       <x:c r="W47" s="10"/>
@@ -3434,7 +3454,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B48" s="12" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C48" s="13"/>
       <x:c r="D48" s="13"/>
@@ -3446,7 +3466,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J48" s="10" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="K48" s="10"/>
       <x:c r="L48" s="10"/>
@@ -3457,7 +3477,7 @@
       <x:c r="Q48" s="10"/>
       <x:c r="R48" s="10"/>
       <x:c r="S48" s="10"/>
-      <x:c r="T48" s="10"/>
+      <x:c r="T48" s="83"/>
       <x:c r="U48" s="10"/>
       <x:c r="V48" s="10"/>
       <x:c r="W48" s="10"/>
@@ -3478,10 +3498,11 @@
       <x:c r="G49" s="23"/>
       <x:c r="H49" s="23"/>
       <x:c r="J49" s="1"/>
+      <x:c r="T49" s="84"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="20" t="s">
-        <x:v>68</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B50" s="20"/>
       <x:c r="C50" s="20"/>
@@ -3501,6 +3522,7 @@
       <x:c r="Q50" s="20"/>
       <x:c r="R50" s="20"/>
       <x:c r="S50" s="20"/>
+      <x:c r="T50" s="84"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="7">
@@ -3524,6 +3546,7 @@
       <x:c r="Q51" s="21"/>
       <x:c r="R51" s="21"/>
       <x:c r="S51" s="22"/>
+      <x:c r="T51" s="84"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="8">
@@ -3547,6 +3570,7 @@
       <x:c r="Q52" s="16"/>
       <x:c r="R52" s="16"/>
       <x:c r="S52" s="17"/>
+      <x:c r="T52" s="84"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="8">
@@ -3570,6 +3594,7 @@
       <x:c r="Q53" s="16"/>
       <x:c r="R53" s="16"/>
       <x:c r="S53" s="17"/>
+      <x:c r="T53" s="84"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="8">
@@ -3593,6 +3618,7 @@
       <x:c r="Q54" s="16"/>
       <x:c r="R54" s="16"/>
       <x:c r="S54" s="17"/>
+      <x:c r="T54" s="84"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="8">
@@ -3616,10 +3642,11 @@
       <x:c r="Q55" s="16"/>
       <x:c r="R55" s="16"/>
       <x:c r="S55" s="17"/>
+      <x:c r="T55" s="84"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="9" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B56" s="18"/>
       <x:c r="C56" s="18"/>
@@ -3639,6 +3666,7 @@
       <x:c r="Q56" s="18"/>
       <x:c r="R56" s="18"/>
       <x:c r="S56" s="19"/>
+      <x:c r="T56" s="84"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3749,7 +3777,6 @@
     <x:mergeCell ref="T40:AC40"/>
     <x:mergeCell ref="T41:AC41"/>
     <x:mergeCell ref="T42:AC42"/>
-    <x:mergeCell ref="A7:T13"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update application form with integrated features
</commit_message>
<xml_diff>
--- a/Prijavnica_ParKING.xlsx
+++ b/Prijavnica_ParKING.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List1" sheetId="1" r:id="R59d29d0622b4439c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List1" sheetId="1" r:id="R73f52b13133f4aac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,6 +226,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -233,7 +237,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -245,7 +249,7 @@
     <x:r>
       <x:rPr>
         <x:b/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -256,7 +260,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -270,6 +274,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -277,7 +285,8 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -286,7 +295,8 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -298,7 +308,8 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -311,6 +322,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -318,7 +333,8 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -327,7 +343,8 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -339,7 +356,8 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -348,7 +366,8 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
         <x:scheme val="minor"/>
@@ -362,6 +381,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Za svaki od pristupa (INI i/ili Windows registar) treba opisati:
 </x:t>
     </x:r>
@@ -369,7 +392,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -380,7 +403,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -395,6 +418,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Za svaki od pristupa (XML i/ili JSON) treba opisati:
 </x:t>
     </x:r>
@@ -402,7 +429,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -414,7 +441,7 @@
     <x:r>
       <x:rPr>
         <x:b/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -424,7 +451,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -440,6 +467,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -447,7 +478,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -460,7 +491,7 @@
     <x:r>
       <x:rPr>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -475,6 +506,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -482,7 +517,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -493,7 +528,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -506,7 +541,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -516,7 +551,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -531,6 +566,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -538,7 +577,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -555,6 +594,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -562,7 +605,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -576,6 +619,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -583,7 +630,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -599,6 +646,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -606,7 +657,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -616,7 +667,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -629,7 +680,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -640,7 +691,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -655,6 +706,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -662,7 +717,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -676,6 +731,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Za svaki korišteni mehanizam međusobnog zaključavanja treba opisati:
 </x:t>
     </x:r>
@@ -683,7 +742,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -697,6 +756,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -704,7 +767,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -714,7 +777,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -727,7 +790,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -741,6 +804,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -748,7 +815,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -766,6 +833,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -773,7 +844,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -788,6 +859,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -795,7 +870,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -809,6 +884,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -816,7 +895,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -831,6 +910,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -838,7 +921,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -852,6 +935,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -859,7 +946,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -875,6 +962,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -882,7 +973,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -896,6 +987,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -903,7 +998,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -914,7 +1009,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -931,6 +1026,10 @@
   </x:si>
   <x:si>
     <x:r>
+      <x:rPr>
+        <x:sz val="1100"/>
+        <x:color rgb="FF000000"/>
+      </x:rPr>
       <x:t xml:space="preserve">Opis treba sadržavati:
 </x:t>
     </x:r>
@@ -938,7 +1037,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -950,7 +1049,7 @@
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -963,7 +1062,7 @@
       <x:rPr>
         <x:b/>
         <x:i/>
-        <x:sz val="11"/>
+        <x:sz val="1100"/>
         <x:color theme="1"/>
         <x:rFont val="Calibri"/>
         <x:family val="2"/>
@@ -1426,7 +1525,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="90">
+  <x:cellXfs count="119">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -1690,6 +1789,91 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="13" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="3">
@@ -2271,7 +2455,7 @@
       <x:c r="AB18" s="15"/>
       <x:c r="AC18" s="15"/>
     </x:row>
-    <x:row r="19" ht="88" customHeight="1">
+    <x:row r="19" ht="92" customHeight="1">
       <x:c r="A19" s="3">
         <x:v>1</x:v>
       </x:c>
@@ -2301,10 +2485,10 @@
       <x:c r="S19" s="14"/>
       <x:c r="T19" s="82" t="str">
         <x:v>Implementirane su tri korisničke klase: User, ParkingSpot i Reservation.
-User: atributi id, username, password_hash, role; metode set_password(), check_password(), is_admin().
-ParkingSpot: atributi id, owner_id, name, location, price_per_hour, description; metode display_price(), is_owned_by().
-Reservation: atributi id, parking_id, user_id, start_time, end_time, status; metode duration_hours(), total_price(), overlaps().
-Klase se koriste kroz SQLAlchemy modele i poslovnu logiku aplikacije.</x:v>
+User: atributi id, username, password_hash, role i api_token; metode set_password(), check_password() i is_admin().
+ParkingSpot: atributi id, owner_id, name, location, price_per_hour, description, photo i photo_mime; metode display_price() i is_owned_by().
+Reservation: atributi id, parking_id, user_id, start_time, end_time i status; metode duration_hours(), total_price() i overlaps().
+Klase se koriste kroz SQLAlchemy modele, relacije i poslovnu logiku aplikacije.</x:v>
       </x:c>
       <x:c r="U19" s="13"/>
       <x:c r="V19" s="13"/>
@@ -2316,7 +2500,7 @@
       <x:c r="AB19" s="13"/>
       <x:c r="AC19" s="14"/>
     </x:row>
-    <x:row r="20" ht="82" customHeight="1">
+    <x:row r="20" ht="118" customHeight="1">
       <x:c r="A20" s="3">
         <x:v>2</x:v>
       </x:c>
@@ -2345,8 +2529,8 @@
       <x:c r="R20" s="34"/>
       <x:c r="S20" s="35"/>
       <x:c r="T20" s="82" t="str">
-        <x:v>Aplikacija sadrži više od tri web forme/dijaloga: prijava, registracija, popis parkinga, dodavanje/uređivanje parkinga, detalji parkinga, rezervacija, moje rezervacije te administratorske forme za korisnike i rezervacije.
-Komunikacija među formama demonstrira se npr. odabirom parkinga na popisu ili detaljima, čime se njegov parking_id prenosi na formu za rezervaciju; nakon spremanja korisnik se preusmjerava na pregled svojih rezervacija.</x:v>
+        <x:v>Aplikacija sadrži više od tri web forme/dijaloga: prijava, registracija, pretraga dostupnih parkinga, dodavanje/uređivanje parkinga, detalji parkinga, rezervacija, moje rezervacije, bilješke te administratorske forme.
+Komunikacija među formama vidljiva je u glavnom toku rezervacije. Na stranici Dostupni parkinzi korisnik odabire lokaciju, početak i završetak termina, opcionalnu maksimalnu cijenu i sortiranje. Odabrani start_time i end_time prenose se kroz Detalji → Rezerviraj, pa su u formi rezervacije već popunjeni. Nakon spremanja korisnik se preusmjerava na Moje rezervacije. Datumsko-vremenska polja koriste 24-satni Flatpickr prikaz.</x:v>
       </x:c>
       <x:c r="U20" s="13"/>
       <x:c r="V20" s="13"/>
@@ -2484,7 +2668,7 @@
       <x:c r="AB23" s="13"/>
       <x:c r="AC23" s="14"/>
     </x:row>
-    <x:row r="24" ht="80" customHeight="1">
+    <x:row r="24" ht="132" customHeight="1">
       <x:c r="A24" s="3">
         <x:v>6</x:v>
       </x:c>
@@ -2513,7 +2697,8 @@
       <x:c r="R24" s="13"/>
       <x:c r="S24" s="14"/>
       <x:c r="T24" s="82" t="str">
-        <x:v>Aplikacija koristi vlastiti binarni format datoteke data/search_history.bin za pohranu niza zapisa povijesti pretraga. Datoteka ima vlastito zaglavlje PKSR, verziju formata i broj zapisa. Svaki binarni zapis sadrži user_id, vrijeme zapisa, maksimalnu cijenu i lokaciju promjenjive duljine. Implementirane su funkcije za zapis cijelog niza u binarnu datoteku i ponovno čitanje zapisa iz tog formata. Binarni sadržaj demonstriran je alatom xxd, pri čemu se vidi zaglavlje PKSR i strukturirani binarni podaci, a ne tekstualni zapis.</x:v>
+        <x:v>Aplikacija koristi vlastiti binarni format data/search_history.bin za stvarnu povijest pretraga parkinga. Kada prijavljeni korisnik na stranici Dostupni parkinzi pokrene valjanu pretragu, kriteriji se automatski spremaju u binarnu datoteku; nema ručnog unosa testnih zapisa.
+Format koristi vlastito zaglavlje PKSR, verziju i broj zapisa. Aktualna verzija 2 za svaki zapis sprema user_id, Unix vrijeme, opcionalnu maksimalnu cijenu te UTF-8 polja promjenjive duljine za lokaciju, početak termina, završetak termina i sortiranje. Stranica Povijest pretraga ponovno čita zapise prijavljenog korisnika i omogućuje akciju Ponovi. binary_store.py može čitati staru verziju 1 i pri sljedećem zapisu migrirati sadržaj u verziju 2.</x:v>
       </x:c>
       <x:c r="U24" s="13"/>
       <x:c r="V24" s="13"/>
@@ -2567,7 +2752,7 @@
       <x:c r="AB25" s="13"/>
       <x:c r="AC25" s="14"/>
     </x:row>
-    <x:row r="26" ht="80" customHeight="1">
+    <x:row r="26" ht="132" customHeight="1">
       <x:c r="A26" s="3">
         <x:v>8</x:v>
       </x:c>
@@ -2596,9 +2781,9 @@
       <x:c r="R26" s="13"/>
       <x:c r="S26" s="14"/>
       <x:c r="T26" s="82" t="str">
-        <x:v>Sortiranje i filtriranje provodi se nad zapisima tablice parking_spots. Parkirna mjesta mogu se filtrirati po lokaciji te sortirati po cijeni uzlazno/silazno i po nazivu.
-Izračunato polje: ukupna cijena rezervacije računa se metodom Reservation.total_price() iz trajanja rezervacije i cijene parkinga po satu.
-Lookup/povezana polja ostvarena su SQLAlchemy relacijama, npr. Reservation.parking za dohvat naziva i lokacije parkinga te ParkingSpot.owner za dohvat vlasnika.</x:v>
+        <x:v>Sortiranje i filtriranje provodi se nad zapisima tablice parking_spots. Parkirna mjesta mogu se filtrirati po lokaciji, maksimalnoj cijeni i vremenskoj dostupnosti te sortirati po cijeni uzlazno/silazno i po nazivu.
+Kod vremenskog kriterija iz rezultata se isključuje parking samo ako ima ACTIVE rezervaciju za koju vrijedi Reservation.start_time &lt; traženi_završetak i Reservation.end_time &gt; traženi_početak. CANCELLED rezervacije ne blokiraju dostupnost, pa parking rezerviran samo dio dana ostaje dostupan u nepreklapajućem terminu.
+Izračunato polje je ukupna cijena rezervacije preko Reservation.total_price(), a lookup/povezana polja ostvarena su ORM relacijama, npr. Reservation.parking i ParkingSpot.owner.</x:v>
       </x:c>
       <x:c r="U26" s="13"/>
       <x:c r="V26" s="13"/>
@@ -2813,7 +2998,7 @@
       <x:c r="AB31" s="10"/>
       <x:c r="AC31" s="10"/>
     </x:row>
-    <x:row r="32" ht="94" customHeight="1">
+    <x:row r="32" ht="116" customHeight="1">
       <x:c r="A32" s="3">
         <x:v>14</x:v>
       </x:c>
@@ -2842,7 +3027,8 @@
       <x:c r="R32" s="10"/>
       <x:c r="S32" s="10"/>
       <x:c r="T32" s="83" t="str">
-        <x:v>Aplikacija demonstrira komunikaciju između dva zasebna procesa. Proces A je Flask aplikacija (run.py) koja pomoću subprocess.run pokreće proces B, zasebnu Python skriptu reservation_worker.py. Proces B čita SQLite bazu i provjerava konzistentnost rezervacija, uključujući neispravne vremenske intervale i preklapanja aktivnih rezervacija. Proces B vraća cjelobrojni izlazni kod: 0 kada je provjera uspješna, 1 kada su pronađeni problemi u podacima, a 2 kod tehničke greške. Proces A čita returncode, stdout i stderr te korisniku prikazuje odgovarajuću poruku. Administratorska stranica Procesi omogućuje i kontroliranu simulaciju greške radi demonstracije nenultog izlaznog koda.</x:v>
+        <x:v>Komunikacija između procesa integrirana je u administratorsko upravljanje rezervacijama. Proces A je glavna Flask aplikacija run.py. Na stranici Admin rezervacije gumb Provjeri rezervacije pomoću subprocess.run pokreće proces B, zasebnu skriptu reservation_worker.py.
+Proces B čita SQLite bazu i provjerava neispravne vremenske intervale te preklapanja ACTIVE rezervacija. Vraća cjelobrojni izlazni kod: 0 kada su podaci ispravni, 1 kada je pronađen problem i 2 kod tehničke greške. Proces A čita returncode, stdout i stderr te rezultat prikazuje izravno iznad tablice rezervacija.</x:v>
       </x:c>
       <x:c r="U32" s="10"/>
       <x:c r="V32" s="10"/>
@@ -3049,7 +3235,7 @@
       <x:c r="AB37" s="10"/>
       <x:c r="AC37" s="10"/>
     </x:row>
-    <x:row r="38" ht="76" customHeight="1">
+    <x:row r="38" ht="84" customHeight="1">
       <x:c r="A38" s="3">
         <x:v>20</x:v>
       </x:c>
@@ -3078,7 +3264,7 @@
       <x:c r="R38" s="10"/>
       <x:c r="S38" s="10"/>
       <x:c r="T38" s="83" t="str">
-        <x:v>Aplikacija se spaja na udaljeni REST web servis Open-Meteo (https://open-meteo.com/). HTTP zahtjevima dohvaća aktualne vremenske podatke za tri lokacije: Zagreb, Samobor i Veliku Goricu. Podaci se koriste na administratorskoj demonstracijskoj stranici Dretve kako bi se prikazali rezultati udaljenog servisa i usporedile performanse sekvencijalnih i paralelnih mrežnih poziva.</x:v>
+        <x:v>Aplikacija se spaja na udaljeni REST web servis Open-Meteo (https://open-meteo.com/). HTTP zahtjevima dohvaća aktualne vremenske podatke za Zagreb, Samobor i Veliku Goricu. Pozivi se koriste na administratorskoj stranici Test → Dretve, gdje se isti mrežni zadaci izvršavaju sekvencijalno i paralelno kako bi se prikazali rezultati udaljenog servisa i usporedilo vrijeme izvršavanja.</x:v>
       </x:c>
       <x:c r="U38" s="10"/>
       <x:c r="V38" s="10"/>
@@ -3172,7 +3358,7 @@
       <x:c r="AB40" s="10"/>
       <x:c r="AC40" s="10"/>
     </x:row>
-    <x:row r="41" ht="76" customHeight="1">
+    <x:row r="41" ht="120" customHeight="1">
       <x:c r="A41" s="3">
         <x:v>23</x:v>
       </x:c>
@@ -3201,7 +3387,8 @@
       <x:c r="R41" s="10"/>
       <x:c r="S41" s="10"/>
       <x:c r="T41" s="83" t="str">
-        <x:v>Aplikacija demonstrira simetrično šifriranje i dešifriranje korisničkih bilješki pomoću algoritma AES-GCM. Za korisnika se generira šifrirana datoteka u direktoriju exports, s vlastitim zaglavljem PKAE i slučajnim nonceom. Šifrirani sadržaj nije čitljiv kao tekst, a aplikacija ga može dešifrirati i ponovno prikazati izvorne bilješke. Lozinke korisnika ne pohranjuju se reverzibilno šifrirane.</x:v>
+        <x:v>Aplikacija koristi simetrično šifriranje i dešifriranje stvarnih korisničkih bilješki pomoću AES-GCM algoritma. Funkcionalnost je integrirana u stranicu Bilješke: korisnik može izraditi šifriranu sigurnosnu kopiju trenutačnih JSON bilješki te otvoriti i dešifrirati postojeću kopiju, nakon čega se sadržaj prikazuje na istoj stranici.
+Kopija se sprema kao exports/notes_user_&lt;id&gt;.aes i koristi vlastito zaglavlje PKAE. AES ključ izvodi se iz aplikacijske tajne i ID-a korisnika, a za svaki izvoz generira se novi slučajni 12-bajtni nonce. Korisničke lozinke nisu reverzibilno šifrirane.</x:v>
       </x:c>
       <x:c r="U41" s="10"/>
       <x:c r="V41" s="10"/>
@@ -3252,7 +3439,7 @@
       <x:c r="AB42" s="10"/>
       <x:c r="AC42" s="10"/>
     </x:row>
-    <x:row r="43" ht="92" customHeight="1">
+    <x:row r="43" ht="124" customHeight="1">
       <x:c r="A43" s="3">
         <x:v>25</x:v>
       </x:c>
@@ -3281,7 +3468,8 @@
       <x:c r="R43" s="10"/>
       <x:c r="S43" s="10"/>
       <x:c r="T43" s="83" t="str">
-        <x:v>Aplikacija demonstrira SHA-256 funkciju sažimanja nad proizvoljnim tekstom. Koristi se promjenjiva sol koja se ne sprema u bazu ni datoteku, nego se deterministički izvodi po pravilu SHA256('ParKING-SHA256-salt:&lt;user_id&gt;:&lt;username&gt;')[0:16], pa različiti korisnici dobivaju različitu sol. Uz sol se koristi i papar iz raspona 0-255. Provjera ispravnosti papra demonstrira se prolaskom kroz cijeli raspon svih 256 mogućih vrijednosti; za testni sažetak pronađena je vrijednost papra 137 i potvrđena ispravnost sažetka.</x:v>
+        <x:v>SHA-256 je integriran u rezervacije kao kontrolni otisak integriteta. Korisnik na stranici Moje rezervacije otvara SHA-256 provjeru za konkretnu rezervaciju. Ulaz u sažimanje čine stvarni podaci rezervacije: ID rezervacije, korisnik, parking, lokacija, početak i završetak, status, cijena po satu i ukupna cijena; promjena bilo kojeg od tih podataka mijenja kontrolni otisak.
+Koristi se promjenjiva sol koja se ne sprema u bazu ni datoteku, nego se deterministički izvodi pravilom SHA256("ParKING-SHA256-salt:&lt;user_id&gt;:&lt;username&gt;")[0:16]. Uz sol se koristi papar iz raspona 0–255. Provjera prolazi kroz svih 256 mogućih vrijednosti papra i uspoređuje kandidat s kontrolnim otiskom.</x:v>
       </x:c>
       <x:c r="U43" s="10"/>
       <x:c r="V43" s="10"/>

</xml_diff>